<commit_message>
Add 36 intraday data points to the tracking list (NIFTY 50 + Next 50)
RK moved TradeX's focus to intraday trading across all NIFTY 50 and NIFTY Next 50 stocks on
2026-10-29. The metric catalog gains eight groups: universe, price levels (previous-day levels,
gap, opening range, pivots/CPR), trend and momentum (VWAP, 5-min EMA/RSI, Supertrend), volume and
liquidity (RVOL, delivery %, depth), F&O-stock derivatives, breadth, fundamentals and intraday
data quality. Every unverified source is marked NOT_VERIFIED. Decision recorded in docs/01 §19.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DmuUzQczL8f1hfzJwmUJTU
</commit_message>
<xml_diff>
--- a/docs/Futures_Tracking_Sheet.xlsx
+++ b/docs/Futures_Tracking_Sheet.xlsx
@@ -632,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="19" min="1" max="1"/>
@@ -1929,37 +1929,711 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="22.5" customHeight="1" s="21"/>
-    <row r="70" ht="22.5" customHeight="1" s="21"/>
-    <row r="71" ht="22.5" customHeight="1" s="21"/>
-    <row r="72" ht="22.5" customHeight="1" s="21"/>
-    <row r="73" ht="22.5" customHeight="1" s="21"/>
-    <row r="74" ht="22.5" customHeight="1" s="21"/>
-    <row r="75" ht="22.5" customHeight="1" s="21"/>
-    <row r="76" ht="22.5" customHeight="1" s="21"/>
-    <row r="77" ht="22.5" customHeight="1" s="21"/>
-    <row r="78" ht="22.5" customHeight="1" s="21"/>
-    <row r="79" ht="22.5" customHeight="1" s="21"/>
-    <row r="80" ht="22.5" customHeight="1" s="21"/>
-    <row r="81" ht="22.5" customHeight="1" s="21"/>
-    <row r="82" ht="22.5" customHeight="1" s="21"/>
+    <row r="69" ht="22.5" customHeight="1" s="21">
+      <c r="A69" s="24" t="inlineStr">
+        <is>
+          <t>Intraday Universe</t>
+        </is>
+      </c>
+      <c r="B69" s="29" t="inlineStr">
+        <is>
+          <t>NIFTY 50 + NIFTY Next 50 constituents</t>
+        </is>
+      </c>
+      <c r="C69" s="30" t="inlineStr">
+        <is>
+          <t>The 100 stocks tracked intraday. Membership changes at NSE's semi-annual rebalancing, so the list is read from NSE, never typed in.</t>
+        </is>
+      </c>
+      <c r="D69" s="31" t="inlineStr">
+        <is>
+          <t>NSE index constituent files (ind_nifty50list.csv, ind_niftynext50list.csv on nsearchives) — NOT_VERIFIED from our server</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22.5" customHeight="1" s="21">
+      <c r="A70" s="28" t="n"/>
+      <c r="B70" s="29" t="inlineStr">
+        <is>
+          <t>Sector / Industry</t>
+        </is>
+      </c>
+      <c r="C70" s="30" t="inlineStr">
+        <is>
+          <t>Each stock's sector, to see whether a move is the stock or its whole sector.</t>
+        </is>
+      </c>
+      <c r="D70" s="31" t="inlineStr">
+        <is>
+          <t>Same NSE constituent files (Industry column) — NOT_VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22.5" customHeight="1" s="21">
+      <c r="A71" s="32" t="n"/>
+      <c r="B71" s="29" t="inlineStr">
+        <is>
+          <t>F&amp;O Eligibility</t>
+        </is>
+      </c>
+      <c r="C71" s="30" t="inlineStr">
+        <is>
+          <t>Whether the stock has futures and options. Only F&amp;O stocks get intraday OI, PCR and basis.</t>
+        </is>
+      </c>
+      <c r="D71" s="31" t="inlineStr">
+        <is>
+          <t>Groww instruments list (refreshed daily) / NSE F&amp;O lot-size file</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22.5" customHeight="1" s="21">
+      <c r="A72" s="24" t="inlineStr">
+        <is>
+          <t>Intraday Price Levels</t>
+        </is>
+      </c>
+      <c r="B72" s="29" t="inlineStr">
+        <is>
+          <t>Previous Day High / Low / Close</t>
+        </is>
+      </c>
+      <c r="C72" s="30" t="inlineStr">
+        <is>
+          <t>Yesterday's high, low and close: the most watched intraday reference levels.</t>
+        </is>
+      </c>
+      <c r="D72" s="31" t="inlineStr">
+        <is>
+          <t>Daily candles (Groww), already stored</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22.5" customHeight="1" s="21">
+      <c r="A73" s="28" t="n"/>
+      <c r="B73" s="29" t="inlineStr">
+        <is>
+          <t>Gap % at Open</t>
+        </is>
+      </c>
+      <c r="C73" s="30" t="inlineStr">
+        <is>
+          <t>Today's open vs yesterday's close, in %. Big gaps often mean news.</t>
+        </is>
+      </c>
+      <c r="D73" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from today's first candle and yesterday's close</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22.5" customHeight="1" s="21">
+      <c r="A74" s="28" t="n"/>
+      <c r="B74" s="29" t="inlineStr">
+        <is>
+          <t>Opening Range (first 15 min)</t>
+        </is>
+      </c>
+      <c r="C74" s="30" t="inlineStr">
+        <is>
+          <t>High and low of 09:15–09:30, and whether price is now above, inside or below it.</t>
+        </is>
+      </c>
+      <c r="D74" s="31" t="inlineStr">
+        <is>
+          <t>Groww 5-min / 15-min candles (interval NOT_VERIFIED in our adapter: only 1h and 1d are wired today)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="22.5" customHeight="1" s="21">
+      <c r="A75" s="28" t="n"/>
+      <c r="B75" s="29" t="inlineStr">
+        <is>
+          <t>Pivot Points (P, R1–R3, S1–S3)</t>
+        </is>
+      </c>
+      <c r="C75" s="30" t="inlineStr">
+        <is>
+          <t>Classic floor-trader levels from yesterday's high, low and close.</t>
+        </is>
+      </c>
+      <c r="D75" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from daily candles</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="22.5" customHeight="1" s="21">
+      <c r="A76" s="28" t="n"/>
+      <c r="B76" s="29" t="inlineStr">
+        <is>
+          <t>Central Pivot Range (CPR) &amp; Width</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="inlineStr">
+        <is>
+          <t>Pivot, top and bottom central levels; a narrow CPR often comes before a trending day.</t>
+        </is>
+      </c>
+      <c r="D76" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from daily candles</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="22.5" customHeight="1" s="21">
+      <c r="A77" s="28" t="n"/>
+      <c r="B77" s="29" t="inlineStr">
+        <is>
+          <t>Day High / Low So Far</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>Today's running high and low, and how far price is from each.</t>
+        </is>
+      </c>
+      <c r="D77" s="31" t="inlineStr">
+        <is>
+          <t>Groww live quote, every collector cycle (already collected for tracked contracts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22.5" customHeight="1" s="21">
+      <c r="A78" s="28" t="n"/>
+      <c r="B78" s="29" t="inlineStr">
+        <is>
+          <t>52-Week High / Low Distance</t>
+        </is>
+      </c>
+      <c r="C78" s="30" t="inlineStr">
+        <is>
+          <t>How far price is from its 1-year high and low, in %.</t>
+        </is>
+      </c>
+      <c r="D78" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from daily candles</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="22.5" customHeight="1" s="21">
+      <c r="A79" s="32" t="n"/>
+      <c r="B79" s="29" t="inlineStr">
+        <is>
+          <t>Circuit Limits</t>
+        </is>
+      </c>
+      <c r="C79" s="30" t="inlineStr">
+        <is>
+          <t>Today's upper and lower price bands, and distance to them (stocks only).</t>
+        </is>
+      </c>
+      <c r="D79" s="31" t="inlineStr">
+        <is>
+          <t>Groww quote (upper/lower circuit fields NOT_VERIFIED) or NSE price-band file — NOT_VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="22.5" customHeight="1" s="21">
+      <c r="A80" s="24" t="inlineStr">
+        <is>
+          <t>Intraday Trend &amp; Momentum</t>
+        </is>
+      </c>
+      <c r="B80" s="29" t="inlineStr">
+        <is>
+          <t>VWAP &amp; Distance from VWAP</t>
+        </is>
+      </c>
+      <c r="C80" s="30" t="inlineStr">
+        <is>
+          <t>Volume-weighted average price since 09:15, and price's distance from it in %. Above VWAP = buyers in control so far.</t>
+        </is>
+      </c>
+      <c r="D80" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from intraday candles (Groww 5-min / 15-min candles (interval NOT_VERIFIED in our adapter: only 1h and 1d are wired today))</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22.5" customHeight="1" s="21">
+      <c r="A81" s="28" t="n"/>
+      <c r="B81" s="29" t="inlineStr">
+        <is>
+          <t>VWAP Bands (±1, ±2 SD)</t>
+        </is>
+      </c>
+      <c r="C81" s="30" t="inlineStr">
+        <is>
+          <t>How stretched price is from VWAP, in standard deviations.</t>
+        </is>
+      </c>
+      <c r="D81" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from intraday candles</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22.5" customHeight="1" s="21">
+      <c r="A82" s="28" t="n"/>
+      <c r="B82" s="29" t="inlineStr">
+        <is>
+          <t>Intraday EMA 9 / 20 (5-min)</t>
+        </is>
+      </c>
+      <c r="C82" s="30" t="inlineStr">
+        <is>
+          <t>Short averages on 5-minute candles: the intraday trend.</t>
+        </is>
+      </c>
+      <c r="D82" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from 5-min candles</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="22.5" customHeight="1" s="21">
+      <c r="A83" s="28" t="n"/>
+      <c r="B83" s="29" t="inlineStr">
+        <is>
+          <t>Intraday RSI 14 (5-min)</t>
+        </is>
+      </c>
+      <c r="C83" s="30" t="inlineStr">
+        <is>
+          <t>Momentum on 5-minute candles.</t>
+        </is>
+      </c>
+      <c r="D83" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from 5-min candles</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22.5" customHeight="1" s="21">
+      <c r="A84" s="28" t="n"/>
+      <c r="B84" s="29" t="inlineStr">
+        <is>
+          <t>Supertrend (15-min, 10, 3)</t>
+        </is>
+      </c>
+      <c r="C84" s="30" t="inlineStr">
+        <is>
+          <t>ATR-based trend line on 15-minute candles, widely used by intraday traders.</t>
+        </is>
+      </c>
+      <c r="D84" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from 15-min candles</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22.5" customHeight="1" s="21">
+      <c r="A85" s="28" t="n"/>
+      <c r="B85" s="29" t="inlineStr">
+        <is>
+          <t>Intraday Range vs Daily ATR</t>
+        </is>
+      </c>
+      <c r="C85" s="30" t="inlineStr">
+        <is>
+          <t>Today's high−low so far as a share of the 14-day ATR: has the day already moved its usual amount?</t>
+        </is>
+      </c>
+      <c r="D85" s="31" t="inlineStr">
+        <is>
+          <t>Calculated (live day range ÷ ATR 14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22.5" customHeight="1" s="21">
+      <c r="A86" s="32" t="n"/>
+      <c r="B86" s="29" t="inlineStr">
+        <is>
+          <t>Relative Strength vs NIFTY (intraday)</t>
+        </is>
+      </c>
+      <c r="C86" s="30" t="inlineStr">
+        <is>
+          <t>Stock's % change today minus NIFTY's: stronger or weaker than the market.</t>
+        </is>
+      </c>
+      <c r="D86" s="31" t="inlineStr">
+        <is>
+          <t>Groww live quote, every collector cycle (already collected for tracked contracts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22.5" customHeight="1" s="21">
+      <c r="A87" s="24" t="inlineStr">
+        <is>
+          <t>Intraday Volume &amp; Liquidity</t>
+        </is>
+      </c>
+      <c r="B87" s="29" t="inlineStr">
+        <is>
+          <t>Relative Volume (RVOL)</t>
+        </is>
+      </c>
+      <c r="C87" s="30" t="inlineStr">
+        <is>
+          <t>Volume so far today vs the average volume by the same time of day over 20 days. Above 1 = unusual interest.</t>
+        </is>
+      </c>
+      <c r="D87" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from intraday candles (Groww 5-min / 15-min candles (interval NOT_VERIFIED in our adapter: only 1h and 1d are wired today))</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22.5" customHeight="1" s="21">
+      <c r="A88" s="28" t="n"/>
+      <c r="B88" s="29" t="inlineStr">
+        <is>
+          <t>Volume Spike (5-min)</t>
+        </is>
+      </c>
+      <c r="C88" s="30" t="inlineStr">
+        <is>
+          <t>A 5-minute candle's volume vs the last 20 candles' average.</t>
+        </is>
+      </c>
+      <c r="D88" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from 5-min candles</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="22.5" customHeight="1" s="21">
+      <c r="A89" s="28" t="n"/>
+      <c r="B89" s="29" t="inlineStr">
+        <is>
+          <t>Delivery % (previous day)</t>
+        </is>
+      </c>
+      <c r="C89" s="30" t="inlineStr">
+        <is>
+          <t>Share of yesterday's traded quantity actually delivered; high delivery = positional buying, low = intraday churn.</t>
+        </is>
+      </c>
+      <c r="D89" s="31" t="inlineStr">
+        <is>
+          <t>NSE daily security-wise delivery file (sec_bhavdata_full) — NOT_VERIFIED from our server</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22.5" customHeight="1" s="21">
+      <c r="A90" s="28" t="n"/>
+      <c r="B90" s="29" t="inlineStr">
+        <is>
+          <t>Bid-Ask Spread &amp; Market Depth</t>
+        </is>
+      </c>
+      <c r="C90" s="30" t="inlineStr">
+        <is>
+          <t>Spread and top-5 bid/ask quantities: how easily you can get in and out.</t>
+        </is>
+      </c>
+      <c r="D90" s="31" t="inlineStr">
+        <is>
+          <t>Groww quote depth fields — NOT_VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22.5" customHeight="1" s="21">
+      <c r="A91" s="32" t="n"/>
+      <c r="B91" s="29" t="inlineStr">
+        <is>
+          <t>Bulk &amp; Block Deals</t>
+        </is>
+      </c>
+      <c r="C91" s="30" t="inlineStr">
+        <is>
+          <t>Large trades disclosed by NSE for the stock, previous day.</t>
+        </is>
+      </c>
+      <c r="D91" s="31" t="inlineStr">
+        <is>
+          <t>NSE bulk/block deal daily files — NOT_VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="22.5" customHeight="1" s="21">
+      <c r="A92" s="24" t="inlineStr">
+        <is>
+          <t>Intraday Derivatives (F&amp;O stocks)</t>
+        </is>
+      </c>
+      <c r="B92" s="29" t="inlineStr">
+        <is>
+          <t>Intraday Futures OI Change</t>
+        </is>
+      </c>
+      <c r="C92" s="30" t="inlineStr">
+        <is>
+          <t>Futures OI change through the day, read with price (long/short build-up by 15-minute block).</t>
+        </is>
+      </c>
+      <c r="D92" s="31" t="inlineStr">
+        <is>
+          <t>Groww quote OI on the near future, every cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22.5" customHeight="1" s="21">
+      <c r="A93" s="28" t="n"/>
+      <c r="B93" s="29" t="inlineStr">
+        <is>
+          <t>Intraday PCR &amp; Strike OI</t>
+        </is>
+      </c>
+      <c r="C93" s="30" t="inlineStr">
+        <is>
+          <t>Put-call ratio and biggest call/put OI strikes during the day, near expiry.</t>
+        </is>
+      </c>
+      <c r="D93" s="31" t="inlineStr">
+        <is>
+          <t>Groww option chain, polled intraday (fields NOT_VERIFIED: tradex.sh chain-fields)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22.5" customHeight="1" s="21">
+      <c r="A94" s="32" t="n"/>
+      <c r="B94" s="29" t="inlineStr">
+        <is>
+          <t>Intraday Futures Basis</t>
+        </is>
+      </c>
+      <c r="C94" s="30" t="inlineStr">
+        <is>
+          <t>Near-future price minus cash price, live.</t>
+        </is>
+      </c>
+      <c r="D94" s="31" t="inlineStr">
+        <is>
+          <t>Groww live quote, every collector cycle (already collected for tracked contracts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22.5" customHeight="1" s="21">
+      <c r="A95" s="24" t="inlineStr">
+        <is>
+          <t>Market Breadth &amp; Context</t>
+        </is>
+      </c>
+      <c r="B95" s="29" t="inlineStr">
+        <is>
+          <t>Advance / Decline (NIFTY 100)</t>
+        </is>
+      </c>
+      <c r="C95" s="30" t="inlineStr">
+        <is>
+          <t>How many of the 100 stocks are up vs down right now: broad strength or a few heavyweights.</t>
+        </is>
+      </c>
+      <c r="D95" s="31" t="inlineStr">
+        <is>
+          <t>Calculated from live quotes of the universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22.5" customHeight="1" s="21">
+      <c r="A96" s="28" t="n"/>
+      <c r="B96" s="29" t="inlineStr">
+        <is>
+          <t>Sector Index Moves</t>
+        </is>
+      </c>
+      <c r="C96" s="30" t="inlineStr">
+        <is>
+          <t>Today's % move of NIFTY Bank, IT, Auto, Pharma, FMCG, Metal etc.</t>
+        </is>
+      </c>
+      <c r="D96" s="31" t="inlineStr">
+        <is>
+          <t>Groww index quotes (sector index symbols NOT_VERIFIED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="22.5" customHeight="1" s="21">
+      <c r="A97" s="28" t="n"/>
+      <c r="B97" s="29" t="inlineStr">
+        <is>
+          <t>India VIX Intraday Change</t>
+        </is>
+      </c>
+      <c r="C97" s="30" t="inlineStr">
+        <is>
+          <t>VIX change since yesterday's close, live.</t>
+        </is>
+      </c>
+      <c r="D97" s="31" t="inlineStr">
+        <is>
+          <t>Groww quote (INDIAVIX, verified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22.5" customHeight="1" s="21">
+      <c r="A98" s="32" t="n"/>
+      <c r="B98" s="29" t="inlineStr">
+        <is>
+          <t>Pre-open Price (09:00–09:08)</t>
+        </is>
+      </c>
+      <c r="C98" s="30" t="inlineStr">
+        <is>
+          <t>NSE pre-open auction price and imbalance before the open.</t>
+        </is>
+      </c>
+      <c r="D98" s="31" t="inlineStr">
+        <is>
+          <t>NSE pre-open data — no confirmed source (Groww NOT_VERIFIED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="22.5" customHeight="1" s="21">
+      <c r="A99" s="24" t="inlineStr">
+        <is>
+          <t>Fundamentals (context, daily)</t>
+        </is>
+      </c>
+      <c r="B99" s="29" t="inlineStr">
+        <is>
+          <t>Market Cap, P/E, P/B</t>
+        </is>
+      </c>
+      <c r="C99" s="30" t="inlineStr">
+        <is>
+          <t>Size and valuation, for context only.</t>
+        </is>
+      </c>
+      <c r="D99" s="31" t="inlineStr">
+        <is>
+          <t>Free source NOT_VERIFIED (NSE quote page is not a stable API); consider a paid data vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="22.5" customHeight="1" s="21">
+      <c r="A100" s="28" t="n"/>
+      <c r="B100" s="29" t="inlineStr">
+        <is>
+          <t>Results / Board Meeting Date</t>
+        </is>
+      </c>
+      <c r="C100" s="30" t="inlineStr">
+        <is>
+          <t>Upcoming results: intraday moves on result days are much larger.</t>
+        </is>
+      </c>
+      <c r="D100" s="31" t="inlineStr">
+        <is>
+          <t>NSE corporate announcements / event calendar — NOT_VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="22.5" customHeight="1" s="21">
+      <c r="A101" s="28" t="n"/>
+      <c r="B101" s="29" t="inlineStr">
+        <is>
+          <t>Dividend / Split / Bonus (ex-dates)</t>
+        </is>
+      </c>
+      <c r="C101" s="30" t="inlineStr">
+        <is>
+          <t>Corporate actions that move the price mechanically on the ex-date.</t>
+        </is>
+      </c>
+      <c r="D101" s="31" t="inlineStr">
+        <is>
+          <t>NSE corporate actions file — NOT_VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="22.5" customHeight="1" s="21">
+      <c r="A102" s="32" t="n"/>
+      <c r="B102" s="29" t="inlineStr">
+        <is>
+          <t>Promoter Holding &amp; Pledge %</t>
+        </is>
+      </c>
+      <c r="C102" s="30" t="inlineStr">
+        <is>
+          <t>Quarterly shareholding; high pledge = forced-selling risk.</t>
+        </is>
+      </c>
+      <c r="D102" s="31" t="inlineStr">
+        <is>
+          <t>NSE shareholding pattern filings (quarterly) — NOT_VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="22.5" customHeight="1" s="21">
+      <c r="A103" s="24" t="inlineStr">
+        <is>
+          <t>Intraday Data Quality</t>
+        </is>
+      </c>
+      <c r="B103" s="29" t="inlineStr">
+        <is>
+          <t>Intraday Candle Completeness</t>
+        </is>
+      </c>
+      <c r="C103" s="30" t="inlineStr">
+        <is>
+          <t>Every 5-minute candle from 09:15 to the latest complete one is present, with valid OHLC.</t>
+        </is>
+      </c>
+      <c r="D103" s="31" t="inlineStr">
+        <is>
+          <t>Calculated during ingestion (system validation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="22.5" customHeight="1" s="21">
+      <c r="A104" s="32" t="n"/>
+      <c r="B104" s="29" t="inlineStr">
+        <is>
+          <t>Quote Freshness (intraday)</t>
+        </is>
+      </c>
+      <c r="C104" s="30" t="inlineStr">
+        <is>
+          <t>Each live quote is from the last collector cycle; older = stale, not used.</t>
+        </is>
+      </c>
+      <c r="D104" s="31" t="inlineStr">
+        <is>
+          <t>Calculated: provider timestamp vs now</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A30:A34"/>
+  <mergeCells count="23">
     <mergeCell ref="A21:A25"/>
     <mergeCell ref="A57:A59"/>
-    <mergeCell ref="A26:A29"/>
     <mergeCell ref="A8:A14"/>
-    <mergeCell ref="A2:A7"/>
-    <mergeCell ref="A60:A64"/>
+    <mergeCell ref="A103:A104"/>
     <mergeCell ref="A47:A51"/>
+    <mergeCell ref="A99:A102"/>
     <mergeCell ref="A65:A68"/>
-    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="A92:A94"/>
     <mergeCell ref="A52:A56"/>
     <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A95:A98"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="A69:A71"/>
+    <mergeCell ref="A60:A64"/>
+    <mergeCell ref="A87:A91"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="A72:A79"/>
     <mergeCell ref="A39:A42"/>
     <mergeCell ref="A35:A38"/>
     <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A80:A86"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>